<commit_message>
Thêm SCR-1505, SCR-1506 (BS-01 đã duyệt) vào ma trận phân quyền và task WEB-061, WEB-062
Ma trận: 10 chức năng mới, vai trò con wf_template_author của AC-01,
ràng buộc bốn mắt khi phát hành mẫu luồng.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KcF1KqAcEP78x5iFSgMFRv
</commit_message>
<xml_diff>
--- a/docs/phan-quyen/ma-tran-phan-quyen.xlsx
+++ b/docs/phan-quyen/ma-tran-phan-quyen.xlsx
@@ -17,10 +17,10 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Chú giải'!$A$1:$C$18</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Vai trò'!$A$1:$I$13</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Ma trận chức năng'!$A$1:$V$157</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Ma trận chức năng'!$A$1:$V$167</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'API'!$A$1:$P$25</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Mức dữ liệu'!$A$1:$F$13</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'SoD'!$A$1:$H$31</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'SoD'!$A$1:$H$33</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -629,12 +629,12 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>156 chức năng, 48 màn hình</t>
+          <t>166 chức năng, 50 màn hình</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>152 chức năng web, 55 ô suy luận</t>
+          <t>162 chức năng web, 58 ô suy luận</t>
         </is>
       </c>
     </row>
@@ -970,7 +970,7 @@
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>realm role `platform_admin`</t>
+          <t>realm role `platform_admin`; vai trò con `wf_template_author` cho đội soạn mẫu luồng (BS-01)</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
@@ -1508,7 +1508,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V157"/>
+  <dimension ref="A1:V167"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -16250,27 +16250,27 @@
     <row r="139">
       <c r="A139" s="9" t="inlineStr">
         <is>
-          <t>QT-16</t>
+          <t>QT-15</t>
         </is>
       </c>
       <c r="B139" s="9" t="inlineStr">
         <is>
-          <t>SCR-1601</t>
+          <t>SCR-1505</t>
         </is>
       </c>
       <c r="C139" s="2" t="inlineStr">
         <is>
-          <t>Bảng điều hành lãnh đạo</t>
+          <t>Thư viện và trình soạn mẫu luồng (nội bộ nền tảng, BS-01)</t>
         </is>
       </c>
       <c r="D139" s="2" t="inlineStr">
         <is>
-          <t>SCR-1601.xem</t>
+          <t>SCR-1505.thu-vien</t>
         </is>
       </c>
       <c r="E139" s="2" t="inlineStr">
         <is>
-          <t>Xem bảng điều hành, so với quý trước, xuất báo cáo</t>
+          <t>Xem thư viện mẫu luồng: phiên bản, trạng thái, số tenant đang dùng, số test</t>
         </is>
       </c>
       <c r="F139" s="9" t="inlineStr">
@@ -16278,9 +16278,9 @@
           <t>Có</t>
         </is>
       </c>
-      <c r="G139" s="9" t="inlineStr">
-        <is>
-          <t>-</t>
+      <c r="G139" s="13" t="inlineStr">
+        <is>
+          <t>R/N</t>
         </is>
       </c>
       <c r="H139" s="9" t="inlineStr">
@@ -16293,14 +16293,14 @@
           <t>-</t>
         </is>
       </c>
-      <c r="J139" s="13" t="inlineStr">
-        <is>
-          <t>R/Cd</t>
-        </is>
-      </c>
-      <c r="K139" s="13" t="inlineStr">
-        <is>
-          <t>R/Đv</t>
+      <c r="J139" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K139" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
       <c r="L139" s="9" t="inlineStr">
@@ -16318,14 +16318,14 @@
           <t>-</t>
         </is>
       </c>
-      <c r="O139" s="9" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P139" s="12" t="inlineStr">
-        <is>
-          <t>R/Cd*</t>
+      <c r="O139" s="12" t="inlineStr">
+        <is>
+          <t>R/N*</t>
+        </is>
+      </c>
+      <c r="P139" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
       <c r="Q139" s="9" t="inlineStr">
@@ -16338,51 +16338,47 @@
           <t>-</t>
         </is>
       </c>
-      <c r="S139" s="2" t="inlineStr">
-        <is>
-          <t>BR-16-01 (lọc theo cây tổ chức)</t>
-        </is>
-      </c>
+      <c r="S139" s="2" t="inlineStr"/>
       <c r="T139" s="2" t="inlineStr">
         <is>
-          <t>`POST /api/v1/analytics/query`, `/api/v1/analytics/reports`</t>
+          <t>`GET /api/v1/workflow/templates`*</t>
         </is>
       </c>
       <c r="U139" s="2" t="inlineStr">
         <is>
-          <t>SCR-1601; TL-01 Phụ lục C (`manager`, `inspector`)</t>
+          <t>BS-01 (đã duyệt 19/10/2026) SCR-1505 Bố cục</t>
         </is>
       </c>
       <c r="V139" s="2" t="inlineStr">
         <is>
-          <t>AC-10 có trong TL-01 và menu hiện tại nhưng không có trong tác nhân SCR-1601.</t>
+          <t>Chỉ người giữ vai trò con `wf_template_author` của AC-01; AC-09 xem để phê duyệt (suy luận). Tenant không thấy màn hình.</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" s="9" t="inlineStr">
         <is>
-          <t>QT-16</t>
+          <t>QT-15</t>
         </is>
       </c>
       <c r="B140" s="9" t="inlineStr">
         <is>
-          <t>SCR-1601</t>
+          <t>SCR-1505</t>
         </is>
       </c>
       <c r="C140" s="2" t="inlineStr">
         <is>
-          <t>Bảng điều hành lãnh đạo</t>
+          <t>Thư viện và trình soạn mẫu luồng (nội bộ nền tảng, BS-01)</t>
         </is>
       </c>
       <c r="D140" s="2" t="inlineStr">
         <is>
-          <t>SCR-1601.nhac</t>
+          <t>SCR-1505.soan</t>
         </is>
       </c>
       <c r="E140" s="2" t="inlineStr">
         <is>
-          <t>Nhắc người chủ trì việc chậm</t>
+          <t>Soạn, sửa mẫu luồng bằng bpmn-js, khai báo tham số; linter bpmnlint chạy ngay trên trình duyệt</t>
         </is>
       </c>
       <c r="F140" s="9" t="inlineStr">
@@ -16390,9 +16386,9 @@
           <t>Có</t>
         </is>
       </c>
-      <c r="G140" s="9" t="inlineStr">
-        <is>
-          <t>-</t>
+      <c r="G140" s="10" t="inlineStr">
+        <is>
+          <t>T/N</t>
         </is>
       </c>
       <c r="H140" s="9" t="inlineStr">
@@ -16405,14 +16401,14 @@
           <t>-</t>
         </is>
       </c>
-      <c r="J140" s="10" t="inlineStr">
-        <is>
-          <t>T/Cd</t>
-        </is>
-      </c>
-      <c r="K140" s="10" t="inlineStr">
-        <is>
-          <t>T/Đv</t>
+      <c r="J140" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K140" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
       <c r="L140" s="9" t="inlineStr">
@@ -16452,45 +16448,49 @@
       </c>
       <c r="S140" s="2" t="inlineStr">
         <is>
-          <t>BR-16-07 (dùng quyền của người bấm)</t>
+          <t>4 quy tắc chống mạng nhện (TL-01), máy chủ chạy lại linter khi lưu</t>
         </is>
       </c>
       <c r="T140" s="2" t="inlineStr">
         <is>
-          <t>`POST /api/v1/tasks/{id}/reminders`</t>
+          <t>`POST/PUT /api/v1/workflow/templates`*</t>
         </is>
       </c>
       <c r="U140" s="2" t="inlineStr">
         <is>
-          <t>SCR-1601</t>
-        </is>
-      </c>
-      <c r="V140" s="2" t="inlineStr"/>
+          <t>BS-01 (đã duyệt 19/10/2026) SCR-1505 Kiểm tra khi soạn</t>
+        </is>
+      </c>
+      <c r="V140" s="2" t="inlineStr">
+        <is>
+          <t>Vai trò `wf_template_author`. Phiên bản HIEU_LUC không sửa được.</t>
+        </is>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="9" t="inlineStr">
         <is>
-          <t>QT-16</t>
+          <t>QT-15</t>
         </is>
       </c>
       <c r="B141" s="9" t="inlineStr">
         <is>
-          <t>SCR-1601</t>
+          <t>SCR-1505</t>
         </is>
       </c>
       <c r="C141" s="2" t="inlineStr">
         <is>
-          <t>Bảng điều hành lãnh đạo</t>
+          <t>Thư viện và trình soạn mẫu luồng (nội bộ nền tảng, BS-01)</t>
         </is>
       </c>
       <c r="D141" s="2" t="inlineStr">
         <is>
-          <t>SCR-1601.giao-lai</t>
+          <t>SCR-1505.chay-test</t>
         </is>
       </c>
       <c r="E141" s="2" t="inlineStr">
         <is>
-          <t>Giao lại nhiệm vụ trong phạm vi</t>
+          <t>Chạy bộ test kịch bản và thử tải rút gọn trên engine kiểm thử riêng</t>
         </is>
       </c>
       <c r="F141" s="9" t="inlineStr">
@@ -16498,9 +16498,9 @@
           <t>Có</t>
         </is>
       </c>
-      <c r="G141" s="9" t="inlineStr">
-        <is>
-          <t>-</t>
+      <c r="G141" s="10" t="inlineStr">
+        <is>
+          <t>T/N</t>
         </is>
       </c>
       <c r="H141" s="9" t="inlineStr">
@@ -16513,14 +16513,14 @@
           <t>-</t>
         </is>
       </c>
-      <c r="J141" s="14" t="inlineStr">
-        <is>
-          <t>T/Cd*</t>
-        </is>
-      </c>
-      <c r="K141" s="10" t="inlineStr">
-        <is>
-          <t>T/Đv</t>
+      <c r="J141" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K141" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
       <c r="L141" s="9" t="inlineStr">
@@ -16560,17 +16560,17 @@
       </c>
       <c r="S141" s="2" t="inlineStr">
         <is>
-          <t>BR-16-07; người bấm có quyền giao</t>
+          <t>≤ 20 câu SQL mỗi lần hoàn thành user task; ≤ 12 user task mỗi nhánh; ≤ 50 phần tử đa thể hiện</t>
         </is>
       </c>
       <c r="T141" s="2" t="inlineStr">
         <is>
-          <t>`POST /api/v1/tasks/{id}/reassign`</t>
+          <t>`POST /api/v1/workflow/templates/{id}/test`* (202 + job)</t>
         </is>
       </c>
       <c r="U141" s="2" t="inlineStr">
         <is>
-          <t>SCR-1601</t>
+          <t>BS-01 (đã duyệt 19/10/2026) SCR-1505 Kiểm thử; Giới hạn tải</t>
         </is>
       </c>
       <c r="V141" s="2" t="inlineStr"/>
@@ -16578,27 +16578,27 @@
     <row r="142">
       <c r="A142" s="9" t="inlineStr">
         <is>
-          <t>QT-16</t>
+          <t>QT-15</t>
         </is>
       </c>
       <c r="B142" s="9" t="inlineStr">
         <is>
-          <t>SCR-1601</t>
+          <t>SCR-1505</t>
         </is>
       </c>
       <c r="C142" s="2" t="inlineStr">
         <is>
-          <t>Bảng điều hành lãnh đạo</t>
+          <t>Thư viện và trình soạn mẫu luồng (nội bộ nền tảng, BS-01)</t>
         </is>
       </c>
       <c r="D142" s="2" t="inlineStr">
         <is>
-          <t>SCR-1601.nguon-ai</t>
+          <t>SCR-1505.de-nghi-phat-hanh</t>
         </is>
       </c>
       <c r="E142" s="2" t="inlineStr">
         <is>
-          <t>Xem dữ liệu AI đã dùng cho tóm tắt</t>
+          <t>Đề nghị phát hành: tạo merge request vào repo mẫu luồng kèm BPMN, tham số, test</t>
         </is>
       </c>
       <c r="F142" s="9" t="inlineStr">
@@ -16606,9 +16606,9 @@
           <t>Có</t>
         </is>
       </c>
-      <c r="G142" s="9" t="inlineStr">
-        <is>
-          <t>-</t>
+      <c r="G142" s="10" t="inlineStr">
+        <is>
+          <t>T/N</t>
         </is>
       </c>
       <c r="H142" s="9" t="inlineStr">
@@ -16621,14 +16621,14 @@
           <t>-</t>
         </is>
       </c>
-      <c r="J142" s="13" t="inlineStr">
-        <is>
-          <t>R/Cd</t>
-        </is>
-      </c>
-      <c r="K142" s="13" t="inlineStr">
-        <is>
-          <t>R/Đv</t>
+      <c r="J142" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K142" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
       <c r="L142" s="9" t="inlineStr">
@@ -16661,20 +16661,24 @@
           <t>-</t>
         </is>
       </c>
-      <c r="R142" s="17" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="S142" s="2" t="inlineStr"/>
+      <c r="R142" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S142" s="2" t="inlineStr">
+        <is>
+          <t>Chỉ khi DAT_KIEM_THU</t>
+        </is>
+      </c>
       <c r="T142" s="2" t="inlineStr">
         <is>
-          <t>`GET /api/v1/ai/suggestions/{id}/sources`</t>
+          <t>`POST /api/v1/workflow/templates/{id}/submit`*</t>
         </is>
       </c>
       <c r="U142" s="2" t="inlineStr">
         <is>
-          <t>SCR-1601</t>
+          <t>BS-01 (đã duyệt 19/10/2026) SCR-1505 Đồng bộ với kho mã</t>
         </is>
       </c>
       <c r="V142" s="2" t="inlineStr"/>
@@ -16682,27 +16686,27 @@
     <row r="143">
       <c r="A143" s="9" t="inlineStr">
         <is>
-          <t>QT-16</t>
+          <t>QT-15</t>
         </is>
       </c>
       <c r="B143" s="9" t="inlineStr">
         <is>
-          <t>SCR-1602</t>
+          <t>SCR-1505</t>
         </is>
       </c>
       <c r="C143" s="2" t="inlineStr">
         <is>
-          <t>Trình dựng dashboard</t>
+          <t>Thư viện và trình soạn mẫu luồng (nội bộ nền tảng, BS-01)</t>
         </is>
       </c>
       <c r="D143" s="2" t="inlineStr">
         <is>
-          <t>SCR-1602.dung</t>
+          <t>SCR-1505.phe-duyet</t>
         </is>
       </c>
       <c r="E143" s="2" t="inlineStr">
         <is>
-          <t>Dựng, xem trước, lưu dashboard</t>
+          <t>Phê duyệt phát hành mẫu luồng (bốn mắt), ký số gói mẫu</t>
         </is>
       </c>
       <c r="F143" s="9" t="inlineStr">
@@ -16725,14 +16729,14 @@
           <t>-</t>
         </is>
       </c>
-      <c r="J143" s="10" t="inlineStr">
-        <is>
-          <t>T/Cd</t>
-        </is>
-      </c>
-      <c r="K143" s="10" t="inlineStr">
-        <is>
-          <t>T/Đv</t>
+      <c r="J143" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K143" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
       <c r="L143" s="9" t="inlineStr">
@@ -16750,9 +16754,9 @@
           <t>-</t>
         </is>
       </c>
-      <c r="O143" s="9" t="inlineStr">
-        <is>
-          <t>-</t>
+      <c r="O143" s="16" t="inlineStr">
+        <is>
+          <t>D/N</t>
         </is>
       </c>
       <c r="P143" s="9" t="inlineStr">
@@ -16772,45 +16776,49 @@
       </c>
       <c r="S143" s="2" t="inlineStr">
         <is>
-          <t>Dữ liệu theo phạm vi của người xem</t>
+          <t>Bốn mắt: người duyệt khác người soạn; AAL2, step-up</t>
         </is>
       </c>
       <c r="T143" s="2" t="inlineStr">
         <is>
-          <t>`PUT /api/v1/analytics/dashboards/{id}`</t>
+          <t>Merge request + `POST /api/v1/workflow/templates/{id}/approve`*</t>
         </is>
       </c>
       <c r="U143" s="2" t="inlineStr">
         <is>
-          <t>SCR-1602 Quyền: mọi `leader`, `manager`</t>
-        </is>
-      </c>
-      <c r="V143" s="2" t="inlineStr"/>
+          <t>BS-01 (đã duyệt 19/10/2026) SCR-1505 Người dùng và quyền</t>
+        </is>
+      </c>
+      <c r="V143" s="2" t="inlineStr">
+        <is>
+          <t>AC-09 ở phạm vi nền tảng là người của đội sản phẩm Viettel, khác AC-09 trong tenant.</t>
+        </is>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="9" t="inlineStr">
         <is>
-          <t>QT-16</t>
+          <t>QT-15</t>
         </is>
       </c>
       <c r="B144" s="9" t="inlineStr">
         <is>
-          <t>SCR-1602</t>
+          <t>SCR-1505</t>
         </is>
       </c>
       <c r="C144" s="2" t="inlineStr">
         <is>
-          <t>Trình dựng dashboard</t>
+          <t>Thư viện và trình soạn mẫu luồng (nội bộ nền tảng, BS-01)</t>
         </is>
       </c>
       <c r="D144" s="2" t="inlineStr">
         <is>
-          <t>SCR-1602.chia-se</t>
+          <t>SCR-1505.trien-khai-cell</t>
         </is>
       </c>
       <c r="E144" s="2" t="inlineStr">
         <is>
-          <t>Chia sẻ dashboard (`RIENG`, `DON_VI`, `TENANT`)</t>
+          <t>Theo dõi saga triển khai cuốn chiếu lên engine từng cell, bù trừ về phiên bản trước</t>
         </is>
       </c>
       <c r="F144" s="9" t="inlineStr">
@@ -16818,9 +16826,9 @@
           <t>Có</t>
         </is>
       </c>
-      <c r="G144" s="9" t="inlineStr">
-        <is>
-          <t>-</t>
+      <c r="G144" s="15" t="inlineStr">
+        <is>
+          <t>X/N</t>
         </is>
       </c>
       <c r="H144" s="9" t="inlineStr">
@@ -16833,14 +16841,14 @@
           <t>-</t>
         </is>
       </c>
-      <c r="J144" s="10" t="inlineStr">
-        <is>
-          <t>T/Cd</t>
-        </is>
-      </c>
-      <c r="K144" s="10" t="inlineStr">
-        <is>
-          <t>T/Đv</t>
+      <c r="J144" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K144" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
       <c r="L144" s="9" t="inlineStr">
@@ -16878,15 +16886,19 @@
           <t>-</t>
         </is>
       </c>
-      <c r="S144" s="2" t="inlineStr"/>
+      <c r="S144" s="2" t="inlineStr">
+        <is>
+          <t>Ngoài giờ cao điểm, không trong 3 ngày cuối kỳ; CELL-NB trước</t>
+        </is>
+      </c>
       <c r="T144" s="2" t="inlineStr">
         <is>
-          <t>`POST /api/v1/analytics/dashboards/{id}/shares`</t>
+          <t>`GET /api/v1/workflow/templates/{id}/rollouts`*</t>
         </is>
       </c>
       <c r="U144" s="2" t="inlineStr">
         <is>
-          <t>SCR-1602; TL-03 `config.dashboard_def.share_scope`</t>
+          <t>BS-01 (đã duyệt 19/10/2026) SCR-1505 Triển khai lên cell; Giới hạn tải</t>
         </is>
       </c>
       <c r="V144" s="2" t="inlineStr"/>
@@ -16894,27 +16906,27 @@
     <row r="145">
       <c r="A145" s="9" t="inlineStr">
         <is>
-          <t>QT-16</t>
+          <t>QT-15</t>
         </is>
       </c>
       <c r="B145" s="9" t="inlineStr">
         <is>
-          <t>SCR-1603</t>
+          <t>SCR-1506</t>
         </is>
       </c>
       <c r="C145" s="2" t="inlineStr">
         <is>
-          <t>Đi xuống tới minh chứng</t>
+          <t>Giám sát tiến trình theo mẫu (BS-01)</t>
         </is>
       </c>
       <c r="D145" s="2" t="inlineStr">
         <is>
-          <t>SCR-1603.xem</t>
+          <t>SCR-1506.xem</t>
         </is>
       </c>
       <c r="E145" s="2" t="inlineStr">
         <is>
-          <t>Xem chuỗi truy vết từ điểm tới minh chứng và ngược lên mục tiêu</t>
+          <t>Xem tiến trình đang chạy theo mẫu, phát hiện tiến trình kẹt</t>
         </is>
       </c>
       <c r="F145" s="9" t="inlineStr">
@@ -16922,14 +16934,14 @@
           <t>Có</t>
         </is>
       </c>
-      <c r="G145" s="9" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H145" s="9" t="inlineStr">
-        <is>
-          <t>-</t>
+      <c r="G145" s="13" t="inlineStr">
+        <is>
+          <t>R/N</t>
+        </is>
+      </c>
+      <c r="H145" s="13" t="inlineStr">
+        <is>
+          <t>R/Tn</t>
         </is>
       </c>
       <c r="I145" s="9" t="inlineStr">
@@ -16937,14 +16949,14 @@
           <t>-</t>
         </is>
       </c>
-      <c r="J145" s="13" t="inlineStr">
-        <is>
-          <t>R/Cd</t>
-        </is>
-      </c>
-      <c r="K145" s="13" t="inlineStr">
-        <is>
-          <t>R/Đv</t>
+      <c r="J145" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K145" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
       <c r="L145" s="9" t="inlineStr">
@@ -16952,9 +16964,9 @@
           <t>-</t>
         </is>
       </c>
-      <c r="M145" s="13" t="inlineStr">
-        <is>
-          <t>R/Cd</t>
+      <c r="M145" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
       <c r="N145" s="9" t="inlineStr">
@@ -16967,9 +16979,9 @@
           <t>-</t>
         </is>
       </c>
-      <c r="P145" s="13" t="inlineStr">
-        <is>
-          <t>R/Cd</t>
+      <c r="P145" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
       <c r="Q145" s="9" t="inlineStr">
@@ -16984,45 +16996,49 @@
       </c>
       <c r="S145" s="2" t="inlineStr">
         <is>
-          <t>Mỗi mắt xích kiểm quyền riêng; MSG-16-06</t>
+          <t>Không truy vấn ACT_* lúc cao điểm</t>
         </is>
       </c>
       <c r="T145" s="2" t="inlineStr">
         <is>
-          <t>`GET /api/v1/analytics/trace/{objectType}/{id}`</t>
+          <t>`GET /api/v1/workflow/instances`* (đọc wf_task_projection)</t>
         </is>
       </c>
       <c r="U145" s="2" t="inlineStr">
         <is>
-          <t>SCR-1603</t>
-        </is>
-      </c>
-      <c r="V145" s="2" t="inlineStr"/>
+          <t>BS-01 (đã duyệt 19/10/2026) SCR-1506</t>
+        </is>
+      </c>
+      <c r="V145" s="2" t="inlineStr">
+        <is>
+          <t>AC-01 xem tổng hợp theo cell.</t>
+        </is>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="9" t="inlineStr">
         <is>
-          <t>QT-16</t>
+          <t>QT-15</t>
         </is>
       </c>
       <c r="B146" s="9" t="inlineStr">
         <is>
-          <t>SCR-1603</t>
+          <t>SCR-1506</t>
         </is>
       </c>
       <c r="C146" s="2" t="inlineStr">
         <is>
-          <t>Đi xuống tới minh chứng</t>
+          <t>Giám sát tiến trình theo mẫu (BS-01)</t>
         </is>
       </c>
       <c r="D146" s="2" t="inlineStr">
         <is>
-          <t>SCR-1603.mo-c2</t>
+          <t>SCR-1506.chuyen-nguoi-xu-ly</t>
         </is>
       </c>
       <c r="E146" s="2" t="inlineStr">
         <is>
-          <t>Mở tệp minh chứng (ghi nhật ký truy cập)</t>
+          <t>Chuyển người xử lý của user task khi cán bộ nghỉ hoặc chuyển công tác</t>
         </is>
       </c>
       <c r="F146" s="9" t="inlineStr">
@@ -17030,14 +17046,14 @@
           <t>Có</t>
         </is>
       </c>
-      <c r="G146" s="9" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H146" s="9" t="inlineStr">
-        <is>
-          <t>-</t>
+      <c r="G146" s="14" t="inlineStr">
+        <is>
+          <t>T/N*</t>
+        </is>
+      </c>
+      <c r="H146" s="10" t="inlineStr">
+        <is>
+          <t>T/Tn</t>
         </is>
       </c>
       <c r="I146" s="9" t="inlineStr">
@@ -17045,14 +17061,14 @@
           <t>-</t>
         </is>
       </c>
-      <c r="J146" s="13" t="inlineStr">
-        <is>
-          <t>R/Cd</t>
-        </is>
-      </c>
-      <c r="K146" s="13" t="inlineStr">
-        <is>
-          <t>R/Đv</t>
+      <c r="J146" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K146" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
       <c r="L146" s="9" t="inlineStr">
@@ -17060,9 +17076,9 @@
           <t>-</t>
         </is>
       </c>
-      <c r="M146" s="13" t="inlineStr">
-        <is>
-          <t>R/Cd</t>
+      <c r="M146" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
       <c r="N146" s="9" t="inlineStr">
@@ -17075,9 +17091,9 @@
           <t>-</t>
         </is>
       </c>
-      <c r="P146" s="13" t="inlineStr">
-        <is>
-          <t>R/Cd</t>
+      <c r="P146" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
       <c r="Q146" s="9" t="inlineStr">
@@ -17092,45 +17108,49 @@
       </c>
       <c r="S146" s="2" t="inlineStr">
         <is>
-          <t>Có quyền C2</t>
+          <t>Ghi sổ cái</t>
         </is>
       </c>
       <c r="T146" s="2" t="inlineStr">
         <is>
-          <t>`GET /api/v1/evidences/{id}/versions/{v}/content`</t>
+          <t>`POST /api/v1/workflow/tasks/{id}/reassign`*</t>
         </is>
       </c>
       <c r="U146" s="2" t="inlineStr">
         <is>
-          <t>SCR-1603</t>
-        </is>
-      </c>
-      <c r="V146" s="2" t="inlineStr"/>
+          <t>BS-01 (đã duyệt 19/10/2026) SCR-1506</t>
+        </is>
+      </c>
+      <c r="V146" s="2" t="inlineStr">
+        <is>
+          <t>AC-01 thực hiện là suy luận; nguồn nêu thao tác chung cho màn hình.</t>
+        </is>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="9" t="inlineStr">
         <is>
-          <t>QT-16</t>
+          <t>QT-15</t>
         </is>
       </c>
       <c r="B147" s="9" t="inlineStr">
         <is>
-          <t>SCR-1603</t>
+          <t>SCR-1506</t>
         </is>
       </c>
       <c r="C147" s="2" t="inlineStr">
         <is>
-          <t>Đi xuống tới minh chứng</t>
+          <t>Giám sát tiến trình theo mẫu (BS-01)</t>
         </is>
       </c>
       <c r="D147" s="2" t="inlineStr">
         <is>
-          <t>SCR-1603.xuat</t>
+          <t>SCR-1506.gia-han-buoc</t>
         </is>
       </c>
       <c r="E147" s="2" t="inlineStr">
         <is>
-          <t>Xuất chuỗi bằng chứng JSON và PDF</t>
+          <t>Gia hạn thời hạn của một bước</t>
         </is>
       </c>
       <c r="F147" s="9" t="inlineStr">
@@ -17138,14 +17158,14 @@
           <t>Có</t>
         </is>
       </c>
-      <c r="G147" s="9" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H147" s="9" t="inlineStr">
-        <is>
-          <t>-</t>
+      <c r="G147" s="14" t="inlineStr">
+        <is>
+          <t>T/N*</t>
+        </is>
+      </c>
+      <c r="H147" s="10" t="inlineStr">
+        <is>
+          <t>T/Tn</t>
         </is>
       </c>
       <c r="I147" s="9" t="inlineStr">
@@ -17153,14 +17173,14 @@
           <t>-</t>
         </is>
       </c>
-      <c r="J147" s="13" t="inlineStr">
-        <is>
-          <t>R/Cd</t>
-        </is>
-      </c>
-      <c r="K147" s="13" t="inlineStr">
-        <is>
-          <t>R/Đv</t>
+      <c r="J147" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K147" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
       <c r="L147" s="9" t="inlineStr">
@@ -17168,9 +17188,9 @@
           <t>-</t>
         </is>
       </c>
-      <c r="M147" s="13" t="inlineStr">
-        <is>
-          <t>R/Cd</t>
+      <c r="M147" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
       <c r="N147" s="9" t="inlineStr">
@@ -17183,9 +17203,9 @@
           <t>-</t>
         </is>
       </c>
-      <c r="P147" s="13" t="inlineStr">
-        <is>
-          <t>R/Cd</t>
+      <c r="P147" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
       <c r="Q147" s="9" t="inlineStr">
@@ -17198,15 +17218,19 @@
           <t>-</t>
         </is>
       </c>
-      <c r="S147" s="2" t="inlineStr"/>
+      <c r="S147" s="2" t="inlineStr">
+        <is>
+          <t>Ghi sổ cái; không sửa biến, không nhảy bước</t>
+        </is>
+      </c>
       <c r="T147" s="2" t="inlineStr">
         <is>
-          <t>`POST /api/v1/analytics/trace/exports` (202)</t>
+          <t>`POST /api/v1/workflow/tasks/{id}/extend`*</t>
         </is>
       </c>
       <c r="U147" s="2" t="inlineStr">
         <is>
-          <t>SCR-1603</t>
+          <t>BS-01 (đã duyệt 19/10/2026) SCR-1506</t>
         </is>
       </c>
       <c r="V147" s="2" t="inlineStr"/>
@@ -17214,27 +17238,27 @@
     <row r="148">
       <c r="A148" s="9" t="inlineStr">
         <is>
-          <t>QT-17</t>
+          <t>QT-15</t>
         </is>
       </c>
       <c r="B148" s="9" t="inlineStr">
         <is>
-          <t>SCR-1701</t>
+          <t>SCR-1506</t>
         </is>
       </c>
       <c r="C148" s="2" t="inlineStr">
         <is>
-          <t>Trợ lý AI soạn OKR và soát KR</t>
+          <t>Giám sát tiến trình theo mẫu (BS-01)</t>
         </is>
       </c>
       <c r="D148" s="2" t="inlineStr">
         <is>
-          <t>SCR-1701.hoi</t>
+          <t>SCR-1506.so-do</t>
         </is>
       </c>
       <c r="E148" s="2" t="inlineStr">
         <is>
-          <t>Hỏi trợ lý AI, nhận gợi ý OKR, cảnh báo KR mơ hồ</t>
+          <t>Xem sơ đồ tiến trình với bước hiện tại</t>
         </is>
       </c>
       <c r="F148" s="9" t="inlineStr">
@@ -17242,14 +17266,14 @@
           <t>Có</t>
         </is>
       </c>
-      <c r="G148" s="9" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H148" s="9" t="inlineStr">
-        <is>
-          <t>-</t>
+      <c r="G148" s="13" t="inlineStr">
+        <is>
+          <t>R/N</t>
+        </is>
+      </c>
+      <c r="H148" s="13" t="inlineStr">
+        <is>
+          <t>R/Tn</t>
         </is>
       </c>
       <c r="I148" s="9" t="inlineStr">
@@ -17262,14 +17286,14 @@
           <t>-</t>
         </is>
       </c>
-      <c r="K148" s="10" t="inlineStr">
-        <is>
-          <t>T/Đv</t>
-        </is>
-      </c>
-      <c r="L148" s="10" t="inlineStr">
-        <is>
-          <t>T/B</t>
+      <c r="K148" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L148" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
       <c r="M148" s="9" t="inlineStr">
@@ -17297,24 +17321,20 @@
           <t>-</t>
         </is>
       </c>
-      <c r="R148" s="17" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="S148" s="2" t="inlineStr">
-        <is>
-          <t>BR-17-03, BR-17-07; MSG-17-02</t>
-        </is>
-      </c>
+      <c r="R148" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S148" s="2" t="inlineStr"/>
       <c r="T148" s="2" t="inlineStr">
         <is>
-          <t>`POST /api/v1/ai/assist/okr`</t>
+          <t>`GET .../diagram` (đã có ở QT-08)</t>
         </is>
       </c>
       <c r="U148" s="2" t="inlineStr">
         <is>
-          <t>SCR-1701 Quyền: người soạn OKR của đơn vị</t>
+          <t>BS-01 (đã duyệt 19/10/2026) SCR-1506</t>
         </is>
       </c>
       <c r="V148" s="2" t="inlineStr"/>
@@ -17322,27 +17342,27 @@
     <row r="149">
       <c r="A149" s="9" t="inlineStr">
         <is>
-          <t>QT-17</t>
+          <t>QT-16</t>
         </is>
       </c>
       <c r="B149" s="9" t="inlineStr">
         <is>
-          <t>SCR-1701</t>
+          <t>SCR-1601</t>
         </is>
       </c>
       <c r="C149" s="2" t="inlineStr">
         <is>
-          <t>Trợ lý AI soạn OKR và soát KR</t>
+          <t>Bảng điều hành lãnh đạo</t>
         </is>
       </c>
       <c r="D149" s="2" t="inlineStr">
         <is>
-          <t>SCR-1701.dung-goi-y</t>
+          <t>SCR-1601.xem</t>
         </is>
       </c>
       <c r="E149" s="2" t="inlineStr">
         <is>
-          <t>Dùng hoặc bỏ gợi ý, lưu nháp, xem lịch sử nháp</t>
+          <t>Xem bảng điều hành, so với quý trước, xuất báo cáo</t>
         </is>
       </c>
       <c r="F149" s="9" t="inlineStr">
@@ -17365,19 +17385,19 @@
           <t>-</t>
         </is>
       </c>
-      <c r="J149" s="9" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K149" s="10" t="inlineStr">
-        <is>
-          <t>T/Đv</t>
-        </is>
-      </c>
-      <c r="L149" s="10" t="inlineStr">
-        <is>
-          <t>T/B</t>
+      <c r="J149" s="13" t="inlineStr">
+        <is>
+          <t>R/Cd</t>
+        </is>
+      </c>
+      <c r="K149" s="13" t="inlineStr">
+        <is>
+          <t>R/Đv</t>
+        </is>
+      </c>
+      <c r="L149" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
       <c r="M149" s="9" t="inlineStr">
@@ -17395,9 +17415,9 @@
           <t>-</t>
         </is>
       </c>
-      <c r="P149" s="9" t="inlineStr">
-        <is>
-          <t>-</t>
+      <c r="P149" s="12" t="inlineStr">
+        <is>
+          <t>R/Cd*</t>
         </is>
       </c>
       <c r="Q149" s="9" t="inlineStr">
@@ -17412,45 +17432,49 @@
       </c>
       <c r="S149" s="2" t="inlineStr">
         <is>
-          <t>BR-02-11, BR-17-08</t>
+          <t>BR-16-01 (lọc theo cây tổ chức)</t>
         </is>
       </c>
       <c r="T149" s="2" t="inlineStr">
         <is>
-          <t>`POST /api/v1/ai/suggestions/{id}/accept`, `PUT /api/v1/okr/objectives/{id}`</t>
+          <t>`POST /api/v1/analytics/query`, `/api/v1/analytics/reports`</t>
         </is>
       </c>
       <c r="U149" s="2" t="inlineStr">
         <is>
-          <t>SCR-1701</t>
-        </is>
-      </c>
-      <c r="V149" s="2" t="inlineStr"/>
+          <t>SCR-1601; TL-01 Phụ lục C (`manager`, `inspector`)</t>
+        </is>
+      </c>
+      <c r="V149" s="2" t="inlineStr">
+        <is>
+          <t>AC-10 có trong TL-01 và menu hiện tại nhưng không có trong tác nhân SCR-1601.</t>
+        </is>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="9" t="inlineStr">
         <is>
-          <t>QT-17</t>
+          <t>QT-16</t>
         </is>
       </c>
       <c r="B150" s="9" t="inlineStr">
         <is>
-          <t>SCR-1701</t>
+          <t>SCR-1601</t>
         </is>
       </c>
       <c r="C150" s="2" t="inlineStr">
         <is>
-          <t>Trợ lý AI soạn OKR và soát KR</t>
+          <t>Bảng điều hành lãnh đạo</t>
         </is>
       </c>
       <c r="D150" s="2" t="inlineStr">
         <is>
-          <t>SCR-1701.trinh</t>
+          <t>SCR-1601.nhac</t>
         </is>
       </c>
       <c r="E150" s="2" t="inlineStr">
         <is>
-          <t>Trình phê duyệt OKR từ trợ lý</t>
+          <t>Nhắc người chủ trì việc chậm</t>
         </is>
       </c>
       <c r="F150" s="9" t="inlineStr">
@@ -17473,9 +17497,9 @@
           <t>-</t>
         </is>
       </c>
-      <c r="J150" s="9" t="inlineStr">
-        <is>
-          <t>-</t>
+      <c r="J150" s="10" t="inlineStr">
+        <is>
+          <t>T/Cd</t>
         </is>
       </c>
       <c r="K150" s="10" t="inlineStr">
@@ -17483,9 +17507,9 @@
           <t>T/Đv</t>
         </is>
       </c>
-      <c r="L150" s="10" t="inlineStr">
-        <is>
-          <t>T/B</t>
+      <c r="L150" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
       <c r="M150" s="9" t="inlineStr">
@@ -17518,15 +17542,19 @@
           <t>-</t>
         </is>
       </c>
-      <c r="S150" s="2" t="inlineStr"/>
+      <c r="S150" s="2" t="inlineStr">
+        <is>
+          <t>BR-16-07 (dùng quyền của người bấm)</t>
+        </is>
+      </c>
       <c r="T150" s="2" t="inlineStr">
         <is>
-          <t>`POST /api/v1/okr/objectives/{id}/submit`</t>
+          <t>`POST /api/v1/tasks/{id}/reminders`</t>
         </is>
       </c>
       <c r="U150" s="2" t="inlineStr">
         <is>
-          <t>SCR-1701</t>
+          <t>SCR-1601</t>
         </is>
       </c>
       <c r="V150" s="2" t="inlineStr"/>
@@ -17534,27 +17562,27 @@
     <row r="151">
       <c r="A151" s="9" t="inlineStr">
         <is>
-          <t>QT-18</t>
+          <t>QT-16</t>
         </is>
       </c>
       <c r="B151" s="9" t="inlineStr">
         <is>
-          <t>SCR-1801</t>
+          <t>SCR-1601</t>
         </is>
       </c>
       <c r="C151" s="2" t="inlineStr">
         <is>
-          <t>Cấu hình giao diện tenant</t>
+          <t>Bảng điều hành lãnh đạo</t>
         </is>
       </c>
       <c r="D151" s="2" t="inlineStr">
         <is>
-          <t>SCR-1801.soan</t>
+          <t>SCR-1601.giao-lai</t>
         </is>
       </c>
       <c r="E151" s="2" t="inlineStr">
         <is>
-          <t>Soạn token, bố cục, chế độ cao tuổi, thêm widget, xem trước</t>
+          <t>Giao lại nhiệm vụ trong phạm vi</t>
         </is>
       </c>
       <c r="F151" s="9" t="inlineStr">
@@ -17567,9 +17595,9 @@
           <t>-</t>
         </is>
       </c>
-      <c r="H151" s="15" t="inlineStr">
-        <is>
-          <t>X/Tn</t>
+      <c r="H151" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
       <c r="I151" s="9" t="inlineStr">
@@ -17577,14 +17605,14 @@
           <t>-</t>
         </is>
       </c>
-      <c r="J151" s="9" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K151" s="9" t="inlineStr">
-        <is>
-          <t>-</t>
+      <c r="J151" s="14" t="inlineStr">
+        <is>
+          <t>T/Cd*</t>
+        </is>
+      </c>
+      <c r="K151" s="10" t="inlineStr">
+        <is>
+          <t>T/Đv</t>
         </is>
       </c>
       <c r="L151" s="9" t="inlineStr">
@@ -17622,15 +17650,19 @@
           <t>-</t>
         </is>
       </c>
-      <c r="S151" s="2" t="inlineStr"/>
+      <c r="S151" s="2" t="inlineStr">
+        <is>
+          <t>BR-16-07; người bấm có quyền giao</t>
+        </is>
+      </c>
       <c r="T151" s="2" t="inlineStr">
         <is>
-          <t>`PUT /api/v1/ui/packs/{id}/versions/{v}`, `GET .../preview`</t>
+          <t>`POST /api/v1/tasks/{id}/reassign`</t>
         </is>
       </c>
       <c r="U151" s="2" t="inlineStr">
         <is>
-          <t>SCR-1801 Quyền: `tenant_admin` của tenant</t>
+          <t>SCR-1601</t>
         </is>
       </c>
       <c r="V151" s="2" t="inlineStr"/>
@@ -17638,27 +17670,27 @@
     <row r="152">
       <c r="A152" s="9" t="inlineStr">
         <is>
-          <t>QT-18</t>
+          <t>QT-16</t>
         </is>
       </c>
       <c r="B152" s="9" t="inlineStr">
         <is>
-          <t>SCR-1801</t>
+          <t>SCR-1601</t>
         </is>
       </c>
       <c r="C152" s="2" t="inlineStr">
         <is>
-          <t>Cấu hình giao diện tenant</t>
+          <t>Bảng điều hành lãnh đạo</t>
         </is>
       </c>
       <c r="D152" s="2" t="inlineStr">
         <is>
-          <t>SCR-1801.gui-duyet</t>
+          <t>SCR-1601.nguon-ai</t>
         </is>
       </c>
       <c r="E152" s="2" t="inlineStr">
         <is>
-          <t>Gửi duyệt UI Pack</t>
+          <t>Xem dữ liệu AI đã dùng cho tóm tắt</t>
         </is>
       </c>
       <c r="F152" s="9" t="inlineStr">
@@ -17671,9 +17703,9 @@
           <t>-</t>
         </is>
       </c>
-      <c r="H152" s="10" t="inlineStr">
-        <is>
-          <t>T/Tn</t>
+      <c r="H152" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
       <c r="I152" s="9" t="inlineStr">
@@ -17681,14 +17713,14 @@
           <t>-</t>
         </is>
       </c>
-      <c r="J152" s="9" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K152" s="9" t="inlineStr">
-        <is>
-          <t>-</t>
+      <c r="J152" s="13" t="inlineStr">
+        <is>
+          <t>R/Cd</t>
+        </is>
+      </c>
+      <c r="K152" s="13" t="inlineStr">
+        <is>
+          <t>R/Đv</t>
         </is>
       </c>
       <c r="L152" s="9" t="inlineStr">
@@ -17721,24 +17753,20 @@
           <t>-</t>
         </is>
       </c>
-      <c r="R152" s="9" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="S152" s="2" t="inlineStr">
-        <is>
-          <t>BR-18-01, BR-18-08</t>
-        </is>
-      </c>
+      <c r="R152" s="17" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="S152" s="2" t="inlineStr"/>
       <c r="T152" s="2" t="inlineStr">
         <is>
-          <t>`POST /api/v1/ui/packs/{id}/versions/{v}/submit`</t>
+          <t>`GET /api/v1/ai/suggestions/{id}/sources`</t>
         </is>
       </c>
       <c r="U152" s="2" t="inlineStr">
         <is>
-          <t>SCR-1801</t>
+          <t>SCR-1601</t>
         </is>
       </c>
       <c r="V152" s="2" t="inlineStr"/>
@@ -17746,27 +17774,27 @@
     <row r="153">
       <c r="A153" s="9" t="inlineStr">
         <is>
-          <t>QT-18</t>
+          <t>QT-16</t>
         </is>
       </c>
       <c r="B153" s="9" t="inlineStr">
         <is>
-          <t>SCR-1801</t>
+          <t>SCR-1602</t>
         </is>
       </c>
       <c r="C153" s="2" t="inlineStr">
         <is>
-          <t>Cấu hình giao diện tenant</t>
+          <t>Trình dựng dashboard</t>
         </is>
       </c>
       <c r="D153" s="2" t="inlineStr">
         <is>
-          <t>SCR-1801.duyet</t>
+          <t>SCR-1602.dung</t>
         </is>
       </c>
       <c r="E153" s="2" t="inlineStr">
         <is>
-          <t>Duyệt và phát hành UI Pack</t>
+          <t>Dựng, xem trước, lưu dashboard</t>
         </is>
       </c>
       <c r="F153" s="9" t="inlineStr">
@@ -17779,9 +17807,9 @@
           <t>-</t>
         </is>
       </c>
-      <c r="H153" s="20" t="inlineStr">
-        <is>
-          <t>D/Tn*</t>
+      <c r="H153" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
       <c r="I153" s="9" t="inlineStr">
@@ -17789,14 +17817,14 @@
           <t>-</t>
         </is>
       </c>
-      <c r="J153" s="9" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K153" s="9" t="inlineStr">
-        <is>
-          <t>-</t>
+      <c r="J153" s="10" t="inlineStr">
+        <is>
+          <t>T/Cd</t>
+        </is>
+      </c>
+      <c r="K153" s="10" t="inlineStr">
+        <is>
+          <t>T/Đv</t>
         </is>
       </c>
       <c r="L153" s="9" t="inlineStr">
@@ -17836,49 +17864,45 @@
       </c>
       <c r="S153" s="2" t="inlineStr">
         <is>
-          <t>Người duyệt khác người soạn; AAL2 (TL-01 Phụ lục C)</t>
+          <t>Dữ liệu theo phạm vi của người xem</t>
         </is>
       </c>
       <c r="T153" s="2" t="inlineStr">
         <is>
-          <t>`POST /api/v1/ui/packs/{id}/versions/{v}/publish`</t>
+          <t>`PUT /api/v1/analytics/dashboards/{id}`</t>
         </is>
       </c>
       <c r="U153" s="2" t="inlineStr">
         <is>
-          <t>SCR-1801 Quyền: người duyệt khác người soạn</t>
-        </is>
-      </c>
-      <c r="V153" s="2" t="inlineStr">
-        <is>
-          <t>Nguồn không nêu vai trò người duyệt; TL-01 ghi `tenant_admin` nên ánh xạ AC-02 khác người soạn là suy luận.</t>
-        </is>
-      </c>
+          <t>SCR-1602 Quyền: mọi `leader`, `manager`</t>
+        </is>
+      </c>
+      <c r="V153" s="2" t="inlineStr"/>
     </row>
     <row r="154">
       <c r="A154" s="9" t="inlineStr">
         <is>
-          <t>QT-18</t>
+          <t>QT-16</t>
         </is>
       </c>
       <c r="B154" s="9" t="inlineStr">
         <is>
-          <t>SCR-1801</t>
+          <t>SCR-1602</t>
         </is>
       </c>
       <c r="C154" s="2" t="inlineStr">
         <is>
-          <t>Cấu hình giao diện tenant</t>
+          <t>Trình dựng dashboard</t>
         </is>
       </c>
       <c r="D154" s="2" t="inlineStr">
         <is>
-          <t>SCR-1801.quay-lui</t>
+          <t>SCR-1602.chia-se</t>
         </is>
       </c>
       <c r="E154" s="2" t="inlineStr">
         <is>
-          <t>Quay lui về phiên bản `THAY_THE` tương thích</t>
+          <t>Chia sẻ dashboard (`RIENG`, `DON_VI`, `TENANT`)</t>
         </is>
       </c>
       <c r="F154" s="9" t="inlineStr">
@@ -17891,9 +17915,9 @@
           <t>-</t>
         </is>
       </c>
-      <c r="H154" s="15" t="inlineStr">
-        <is>
-          <t>X/Tn</t>
+      <c r="H154" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
       <c r="I154" s="9" t="inlineStr">
@@ -17901,14 +17925,14 @@
           <t>-</t>
         </is>
       </c>
-      <c r="J154" s="9" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K154" s="9" t="inlineStr">
-        <is>
-          <t>-</t>
+      <c r="J154" s="10" t="inlineStr">
+        <is>
+          <t>T/Cd</t>
+        </is>
+      </c>
+      <c r="K154" s="10" t="inlineStr">
+        <is>
+          <t>T/Đv</t>
         </is>
       </c>
       <c r="L154" s="9" t="inlineStr">
@@ -17946,19 +17970,15 @@
           <t>-</t>
         </is>
       </c>
-      <c r="S154" s="2" t="inlineStr">
-        <is>
-          <t>BR-18-10; MSG-18-04</t>
-        </is>
-      </c>
+      <c r="S154" s="2" t="inlineStr"/>
       <c r="T154" s="2" t="inlineStr">
         <is>
-          <t>`POST /api/v1/ui/packs/{id}/versions/{v}/activate`</t>
+          <t>`POST /api/v1/analytics/dashboards/{id}/shares`</t>
         </is>
       </c>
       <c r="U154" s="2" t="inlineStr">
         <is>
-          <t>SCR-1801</t>
+          <t>SCR-1602; TL-03 `config.dashboard_def.share_scope`</t>
         </is>
       </c>
       <c r="V154" s="2" t="inlineStr"/>
@@ -17966,27 +17986,27 @@
     <row r="155">
       <c r="A155" s="9" t="inlineStr">
         <is>
-          <t>QT-18</t>
+          <t>QT-16</t>
         </is>
       </c>
       <c r="B155" s="9" t="inlineStr">
         <is>
-          <t>SCR-1802</t>
+          <t>SCR-1603</t>
         </is>
       </c>
       <c r="C155" s="2" t="inlineStr">
         <is>
-          <t>Trình dựng biểu mẫu động</t>
+          <t>Đi xuống tới minh chứng</t>
         </is>
       </c>
       <c r="D155" s="2" t="inlineStr">
         <is>
-          <t>SCR-1802.dung</t>
+          <t>SCR-1603.xem</t>
         </is>
       </c>
       <c r="E155" s="2" t="inlineStr">
         <is>
-          <t>Dựng biểu mẫu, lưu nháp, chạy bộ test biểu mẫu</t>
+          <t>Xem chuỗi truy vết từ điểm tới minh chứng và ngược lên mục tiêu</t>
         </is>
       </c>
       <c r="F155" s="9" t="inlineStr">
@@ -17999,24 +18019,24 @@
           <t>-</t>
         </is>
       </c>
-      <c r="H155" s="15" t="inlineStr">
-        <is>
-          <t>X/Tn</t>
-        </is>
-      </c>
-      <c r="I155" s="10" t="inlineStr">
-        <is>
-          <t>T/Tn</t>
-        </is>
-      </c>
-      <c r="J155" s="9" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K155" s="9" t="inlineStr">
-        <is>
-          <t>-</t>
+      <c r="H155" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I155" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J155" s="13" t="inlineStr">
+        <is>
+          <t>R/Cd</t>
+        </is>
+      </c>
+      <c r="K155" s="13" t="inlineStr">
+        <is>
+          <t>R/Đv</t>
         </is>
       </c>
       <c r="L155" s="9" t="inlineStr">
@@ -18024,9 +18044,9 @@
           <t>-</t>
         </is>
       </c>
-      <c r="M155" s="9" t="inlineStr">
-        <is>
-          <t>-</t>
+      <c r="M155" s="13" t="inlineStr">
+        <is>
+          <t>R/Cd</t>
         </is>
       </c>
       <c r="N155" s="9" t="inlineStr">
@@ -18039,9 +18059,9 @@
           <t>-</t>
         </is>
       </c>
-      <c r="P155" s="9" t="inlineStr">
-        <is>
-          <t>-</t>
+      <c r="P155" s="13" t="inlineStr">
+        <is>
+          <t>R/Cd</t>
         </is>
       </c>
       <c r="Q155" s="9" t="inlineStr">
@@ -18056,17 +18076,17 @@
       </c>
       <c r="S155" s="2" t="inlineStr">
         <is>
-          <t>BR-18-04, BR-18-05, BR-18-06, BR-18-11</t>
+          <t>Mỗi mắt xích kiểm quyền riêng; MSG-16-06</t>
         </is>
       </c>
       <c r="T155" s="2" t="inlineStr">
         <is>
-          <t>`PUT /api/v1/ui/forms/{key}/versions/{v}`, `.../test-runs`</t>
+          <t>`GET /api/v1/analytics/trace/{objectType}/{id}`</t>
         </is>
       </c>
       <c r="U155" s="2" t="inlineStr">
         <is>
-          <t>SCR-1802 Quyền: `tenant_admin`; AC-03 khi biểu mẫu gắn Policy Pack</t>
+          <t>SCR-1603</t>
         </is>
       </c>
       <c r="V155" s="2" t="inlineStr"/>
@@ -18074,27 +18094,27 @@
     <row r="156">
       <c r="A156" s="9" t="inlineStr">
         <is>
-          <t>QT-18</t>
+          <t>QT-16</t>
         </is>
       </c>
       <c r="B156" s="9" t="inlineStr">
         <is>
-          <t>SCR-1802</t>
+          <t>SCR-1603</t>
         </is>
       </c>
       <c r="C156" s="2" t="inlineStr">
         <is>
-          <t>Trình dựng biểu mẫu động</t>
+          <t>Đi xuống tới minh chứng</t>
         </is>
       </c>
       <c r="D156" s="2" t="inlineStr">
         <is>
-          <t>SCR-1802.dua-vao-pack</t>
+          <t>SCR-1603.mo-c2</t>
         </is>
       </c>
       <c r="E156" s="2" t="inlineStr">
         <is>
-          <t>Đưa biểu mẫu vào UI Pack nháp</t>
+          <t>Mở tệp minh chứng (ghi nhật ký truy cập)</t>
         </is>
       </c>
       <c r="F156" s="9" t="inlineStr">
@@ -18107,9 +18127,9 @@
           <t>-</t>
         </is>
       </c>
-      <c r="H156" s="15" t="inlineStr">
-        <is>
-          <t>X/Tn</t>
+      <c r="H156" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
       <c r="I156" s="9" t="inlineStr">
@@ -18117,14 +18137,14 @@
           <t>-</t>
         </is>
       </c>
-      <c r="J156" s="9" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K156" s="9" t="inlineStr">
-        <is>
-          <t>-</t>
+      <c r="J156" s="13" t="inlineStr">
+        <is>
+          <t>R/Cd</t>
+        </is>
+      </c>
+      <c r="K156" s="13" t="inlineStr">
+        <is>
+          <t>R/Đv</t>
         </is>
       </c>
       <c r="L156" s="9" t="inlineStr">
@@ -18132,9 +18152,9 @@
           <t>-</t>
         </is>
       </c>
-      <c r="M156" s="9" t="inlineStr">
-        <is>
-          <t>-</t>
+      <c r="M156" s="13" t="inlineStr">
+        <is>
+          <t>R/Cd</t>
         </is>
       </c>
       <c r="N156" s="9" t="inlineStr">
@@ -18147,9 +18167,9 @@
           <t>-</t>
         </is>
       </c>
-      <c r="P156" s="9" t="inlineStr">
-        <is>
-          <t>-</t>
+      <c r="P156" s="13" t="inlineStr">
+        <is>
+          <t>R/Cd</t>
         </is>
       </c>
       <c r="Q156" s="9" t="inlineStr">
@@ -18162,15 +18182,19 @@
           <t>-</t>
         </is>
       </c>
-      <c r="S156" s="2" t="inlineStr"/>
+      <c r="S156" s="2" t="inlineStr">
+        <is>
+          <t>Có quyền C2</t>
+        </is>
+      </c>
       <c r="T156" s="2" t="inlineStr">
         <is>
-          <t>`POST /api/v1/ui/packs/{id}/versions/{v}/forms`</t>
+          <t>`GET /api/v1/evidences/{id}/versions/{v}/content`</t>
         </is>
       </c>
       <c r="U156" s="2" t="inlineStr">
         <is>
-          <t>SCR-1802</t>
+          <t>SCR-1603</t>
         </is>
       </c>
       <c r="V156" s="2" t="inlineStr"/>
@@ -18178,32 +18202,32 @@
     <row r="157">
       <c r="A157" s="9" t="inlineStr">
         <is>
-          <t>QT-18</t>
+          <t>QT-16</t>
         </is>
       </c>
       <c r="B157" s="9" t="inlineStr">
         <is>
-          <t>SCR-1803</t>
+          <t>SCR-1603</t>
         </is>
       </c>
       <c r="C157" s="2" t="inlineStr">
         <is>
-          <t>Chế độ Đảng viên cao tuổi (di động)</t>
+          <t>Đi xuống tới minh chứng</t>
         </is>
       </c>
       <c r="D157" s="2" t="inlineStr">
         <is>
-          <t>SCR-1803.dd</t>
+          <t>SCR-1603.xuat</t>
         </is>
       </c>
       <c r="E157" s="2" t="inlineStr">
         <is>
-          <t>[Di động] Chế độ cao tuổi: xác nhận sinh hoạt, tự đánh giá rút gọn, nhập giọng nói</t>
+          <t>Xuất chuỗi bằng chứng JSON và PDF</t>
         </is>
       </c>
       <c r="F157" s="9" t="inlineStr">
         <is>
-          <t>Di động</t>
+          <t>Có</t>
         </is>
       </c>
       <c r="G157" s="9" t="inlineStr">
@@ -18221,24 +18245,24 @@
           <t>-</t>
         </is>
       </c>
-      <c r="J157" s="9" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K157" s="9" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L157" s="10" t="inlineStr">
-        <is>
-          <t>T/B</t>
-        </is>
-      </c>
-      <c r="M157" s="9" t="inlineStr">
-        <is>
-          <t>-</t>
+      <c r="J157" s="13" t="inlineStr">
+        <is>
+          <t>R/Cd</t>
+        </is>
+      </c>
+      <c r="K157" s="13" t="inlineStr">
+        <is>
+          <t>R/Đv</t>
+        </is>
+      </c>
+      <c r="L157" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M157" s="13" t="inlineStr">
+        <is>
+          <t>R/Cd</t>
         </is>
       </c>
       <c r="N157" s="9" t="inlineStr">
@@ -18251,9 +18275,9 @@
           <t>-</t>
         </is>
       </c>
-      <c r="P157" s="9" t="inlineStr">
-        <is>
-          <t>-</t>
+      <c r="P157" s="13" t="inlineStr">
+        <is>
+          <t>R/Cd</t>
         </is>
       </c>
       <c r="Q157" s="9" t="inlineStr">
@@ -18261,26 +18285,1094 @@
           <t>-</t>
         </is>
       </c>
-      <c r="R157" s="18" t="inlineStr">
-        <is>
-          <t>A*</t>
+      <c r="R157" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
       <c r="S157" s="2" t="inlineStr"/>
       <c r="T157" s="2" t="inlineStr">
         <is>
+          <t>`POST /api/v1/analytics/trace/exports` (202)</t>
+        </is>
+      </c>
+      <c r="U157" s="2" t="inlineStr">
+        <is>
+          <t>SCR-1603</t>
+        </is>
+      </c>
+      <c r="V157" s="2" t="inlineStr"/>
+    </row>
+    <row r="158">
+      <c r="A158" s="9" t="inlineStr">
+        <is>
+          <t>QT-17</t>
+        </is>
+      </c>
+      <c r="B158" s="9" t="inlineStr">
+        <is>
+          <t>SCR-1701</t>
+        </is>
+      </c>
+      <c r="C158" s="2" t="inlineStr">
+        <is>
+          <t>Trợ lý AI soạn OKR và soát KR</t>
+        </is>
+      </c>
+      <c r="D158" s="2" t="inlineStr">
+        <is>
+          <t>SCR-1701.hoi</t>
+        </is>
+      </c>
+      <c r="E158" s="2" t="inlineStr">
+        <is>
+          <t>Hỏi trợ lý AI, nhận gợi ý OKR, cảnh báo KR mơ hồ</t>
+        </is>
+      </c>
+      <c r="F158" s="9" t="inlineStr">
+        <is>
+          <t>Có</t>
+        </is>
+      </c>
+      <c r="G158" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H158" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I158" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J158" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K158" s="10" t="inlineStr">
+        <is>
+          <t>T/Đv</t>
+        </is>
+      </c>
+      <c r="L158" s="10" t="inlineStr">
+        <is>
+          <t>T/B</t>
+        </is>
+      </c>
+      <c r="M158" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N158" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O158" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P158" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q158" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R158" s="17" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="S158" s="2" t="inlineStr">
+        <is>
+          <t>BR-17-03, BR-17-07; MSG-17-02</t>
+        </is>
+      </c>
+      <c r="T158" s="2" t="inlineStr">
+        <is>
+          <t>`POST /api/v1/ai/assist/okr`</t>
+        </is>
+      </c>
+      <c r="U158" s="2" t="inlineStr">
+        <is>
+          <t>SCR-1701 Quyền: người soạn OKR của đơn vị</t>
+        </is>
+      </c>
+      <c r="V158" s="2" t="inlineStr"/>
+    </row>
+    <row r="159">
+      <c r="A159" s="9" t="inlineStr">
+        <is>
+          <t>QT-17</t>
+        </is>
+      </c>
+      <c r="B159" s="9" t="inlineStr">
+        <is>
+          <t>SCR-1701</t>
+        </is>
+      </c>
+      <c r="C159" s="2" t="inlineStr">
+        <is>
+          <t>Trợ lý AI soạn OKR và soát KR</t>
+        </is>
+      </c>
+      <c r="D159" s="2" t="inlineStr">
+        <is>
+          <t>SCR-1701.dung-goi-y</t>
+        </is>
+      </c>
+      <c r="E159" s="2" t="inlineStr">
+        <is>
+          <t>Dùng hoặc bỏ gợi ý, lưu nháp, xem lịch sử nháp</t>
+        </is>
+      </c>
+      <c r="F159" s="9" t="inlineStr">
+        <is>
+          <t>Có</t>
+        </is>
+      </c>
+      <c r="G159" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H159" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I159" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J159" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K159" s="10" t="inlineStr">
+        <is>
+          <t>T/Đv</t>
+        </is>
+      </c>
+      <c r="L159" s="10" t="inlineStr">
+        <is>
+          <t>T/B</t>
+        </is>
+      </c>
+      <c r="M159" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N159" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O159" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P159" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q159" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R159" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S159" s="2" t="inlineStr">
+        <is>
+          <t>BR-02-11, BR-17-08</t>
+        </is>
+      </c>
+      <c r="T159" s="2" t="inlineStr">
+        <is>
+          <t>`POST /api/v1/ai/suggestions/{id}/accept`, `PUT /api/v1/okr/objectives/{id}`</t>
+        </is>
+      </c>
+      <c r="U159" s="2" t="inlineStr">
+        <is>
+          <t>SCR-1701</t>
+        </is>
+      </c>
+      <c r="V159" s="2" t="inlineStr"/>
+    </row>
+    <row r="160">
+      <c r="A160" s="9" t="inlineStr">
+        <is>
+          <t>QT-17</t>
+        </is>
+      </c>
+      <c r="B160" s="9" t="inlineStr">
+        <is>
+          <t>SCR-1701</t>
+        </is>
+      </c>
+      <c r="C160" s="2" t="inlineStr">
+        <is>
+          <t>Trợ lý AI soạn OKR và soát KR</t>
+        </is>
+      </c>
+      <c r="D160" s="2" t="inlineStr">
+        <is>
+          <t>SCR-1701.trinh</t>
+        </is>
+      </c>
+      <c r="E160" s="2" t="inlineStr">
+        <is>
+          <t>Trình phê duyệt OKR từ trợ lý</t>
+        </is>
+      </c>
+      <c r="F160" s="9" t="inlineStr">
+        <is>
+          <t>Có</t>
+        </is>
+      </c>
+      <c r="G160" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H160" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I160" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J160" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K160" s="10" t="inlineStr">
+        <is>
+          <t>T/Đv</t>
+        </is>
+      </c>
+      <c r="L160" s="10" t="inlineStr">
+        <is>
+          <t>T/B</t>
+        </is>
+      </c>
+      <c r="M160" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N160" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O160" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P160" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q160" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R160" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S160" s="2" t="inlineStr"/>
+      <c r="T160" s="2" t="inlineStr">
+        <is>
+          <t>`POST /api/v1/okr/objectives/{id}/submit`</t>
+        </is>
+      </c>
+      <c r="U160" s="2" t="inlineStr">
+        <is>
+          <t>SCR-1701</t>
+        </is>
+      </c>
+      <c r="V160" s="2" t="inlineStr"/>
+    </row>
+    <row r="161">
+      <c r="A161" s="9" t="inlineStr">
+        <is>
+          <t>QT-18</t>
+        </is>
+      </c>
+      <c r="B161" s="9" t="inlineStr">
+        <is>
+          <t>SCR-1801</t>
+        </is>
+      </c>
+      <c r="C161" s="2" t="inlineStr">
+        <is>
+          <t>Cấu hình giao diện tenant</t>
+        </is>
+      </c>
+      <c r="D161" s="2" t="inlineStr">
+        <is>
+          <t>SCR-1801.soan</t>
+        </is>
+      </c>
+      <c r="E161" s="2" t="inlineStr">
+        <is>
+          <t>Soạn token, bố cục, chế độ cao tuổi, thêm widget, xem trước</t>
+        </is>
+      </c>
+      <c r="F161" s="9" t="inlineStr">
+        <is>
+          <t>Có</t>
+        </is>
+      </c>
+      <c r="G161" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H161" s="15" t="inlineStr">
+        <is>
+          <t>X/Tn</t>
+        </is>
+      </c>
+      <c r="I161" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J161" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K161" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L161" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M161" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N161" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O161" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P161" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q161" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R161" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S161" s="2" t="inlineStr"/>
+      <c r="T161" s="2" t="inlineStr">
+        <is>
+          <t>`PUT /api/v1/ui/packs/{id}/versions/{v}`, `GET .../preview`</t>
+        </is>
+      </c>
+      <c r="U161" s="2" t="inlineStr">
+        <is>
+          <t>SCR-1801 Quyền: `tenant_admin` của tenant</t>
+        </is>
+      </c>
+      <c r="V161" s="2" t="inlineStr"/>
+    </row>
+    <row r="162">
+      <c r="A162" s="9" t="inlineStr">
+        <is>
+          <t>QT-18</t>
+        </is>
+      </c>
+      <c r="B162" s="9" t="inlineStr">
+        <is>
+          <t>SCR-1801</t>
+        </is>
+      </c>
+      <c r="C162" s="2" t="inlineStr">
+        <is>
+          <t>Cấu hình giao diện tenant</t>
+        </is>
+      </c>
+      <c r="D162" s="2" t="inlineStr">
+        <is>
+          <t>SCR-1801.gui-duyet</t>
+        </is>
+      </c>
+      <c r="E162" s="2" t="inlineStr">
+        <is>
+          <t>Gửi duyệt UI Pack</t>
+        </is>
+      </c>
+      <c r="F162" s="9" t="inlineStr">
+        <is>
+          <t>Có</t>
+        </is>
+      </c>
+      <c r="G162" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H162" s="10" t="inlineStr">
+        <is>
+          <t>T/Tn</t>
+        </is>
+      </c>
+      <c r="I162" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J162" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K162" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L162" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M162" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N162" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O162" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P162" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q162" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R162" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S162" s="2" t="inlineStr">
+        <is>
+          <t>BR-18-01, BR-18-08</t>
+        </is>
+      </c>
+      <c r="T162" s="2" t="inlineStr">
+        <is>
+          <t>`POST /api/v1/ui/packs/{id}/versions/{v}/submit`</t>
+        </is>
+      </c>
+      <c r="U162" s="2" t="inlineStr">
+        <is>
+          <t>SCR-1801</t>
+        </is>
+      </c>
+      <c r="V162" s="2" t="inlineStr"/>
+    </row>
+    <row r="163">
+      <c r="A163" s="9" t="inlineStr">
+        <is>
+          <t>QT-18</t>
+        </is>
+      </c>
+      <c r="B163" s="9" t="inlineStr">
+        <is>
+          <t>SCR-1801</t>
+        </is>
+      </c>
+      <c r="C163" s="2" t="inlineStr">
+        <is>
+          <t>Cấu hình giao diện tenant</t>
+        </is>
+      </c>
+      <c r="D163" s="2" t="inlineStr">
+        <is>
+          <t>SCR-1801.duyet</t>
+        </is>
+      </c>
+      <c r="E163" s="2" t="inlineStr">
+        <is>
+          <t>Duyệt và phát hành UI Pack</t>
+        </is>
+      </c>
+      <c r="F163" s="9" t="inlineStr">
+        <is>
+          <t>Có</t>
+        </is>
+      </c>
+      <c r="G163" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H163" s="20" t="inlineStr">
+        <is>
+          <t>D/Tn*</t>
+        </is>
+      </c>
+      <c r="I163" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J163" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K163" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L163" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M163" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N163" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O163" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P163" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q163" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R163" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S163" s="2" t="inlineStr">
+        <is>
+          <t>Người duyệt khác người soạn; AAL2 (TL-01 Phụ lục C)</t>
+        </is>
+      </c>
+      <c r="T163" s="2" t="inlineStr">
+        <is>
+          <t>`POST /api/v1/ui/packs/{id}/versions/{v}/publish`</t>
+        </is>
+      </c>
+      <c r="U163" s="2" t="inlineStr">
+        <is>
+          <t>SCR-1801 Quyền: người duyệt khác người soạn</t>
+        </is>
+      </c>
+      <c r="V163" s="2" t="inlineStr">
+        <is>
+          <t>Nguồn không nêu vai trò người duyệt; TL-01 ghi `tenant_admin` nên ánh xạ AC-02 khác người soạn là suy luận.</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" s="9" t="inlineStr">
+        <is>
+          <t>QT-18</t>
+        </is>
+      </c>
+      <c r="B164" s="9" t="inlineStr">
+        <is>
+          <t>SCR-1801</t>
+        </is>
+      </c>
+      <c r="C164" s="2" t="inlineStr">
+        <is>
+          <t>Cấu hình giao diện tenant</t>
+        </is>
+      </c>
+      <c r="D164" s="2" t="inlineStr">
+        <is>
+          <t>SCR-1801.quay-lui</t>
+        </is>
+      </c>
+      <c r="E164" s="2" t="inlineStr">
+        <is>
+          <t>Quay lui về phiên bản `THAY_THE` tương thích</t>
+        </is>
+      </c>
+      <c r="F164" s="9" t="inlineStr">
+        <is>
+          <t>Có</t>
+        </is>
+      </c>
+      <c r="G164" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H164" s="15" t="inlineStr">
+        <is>
+          <t>X/Tn</t>
+        </is>
+      </c>
+      <c r="I164" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J164" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K164" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L164" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M164" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N164" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O164" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P164" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q164" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R164" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S164" s="2" t="inlineStr">
+        <is>
+          <t>BR-18-10; MSG-18-04</t>
+        </is>
+      </c>
+      <c r="T164" s="2" t="inlineStr">
+        <is>
+          <t>`POST /api/v1/ui/packs/{id}/versions/{v}/activate`</t>
+        </is>
+      </c>
+      <c r="U164" s="2" t="inlineStr">
+        <is>
+          <t>SCR-1801</t>
+        </is>
+      </c>
+      <c r="V164" s="2" t="inlineStr"/>
+    </row>
+    <row r="165">
+      <c r="A165" s="9" t="inlineStr">
+        <is>
+          <t>QT-18</t>
+        </is>
+      </c>
+      <c r="B165" s="9" t="inlineStr">
+        <is>
+          <t>SCR-1802</t>
+        </is>
+      </c>
+      <c r="C165" s="2" t="inlineStr">
+        <is>
+          <t>Trình dựng biểu mẫu động</t>
+        </is>
+      </c>
+      <c r="D165" s="2" t="inlineStr">
+        <is>
+          <t>SCR-1802.dung</t>
+        </is>
+      </c>
+      <c r="E165" s="2" t="inlineStr">
+        <is>
+          <t>Dựng biểu mẫu, lưu nháp, chạy bộ test biểu mẫu</t>
+        </is>
+      </c>
+      <c r="F165" s="9" t="inlineStr">
+        <is>
+          <t>Có</t>
+        </is>
+      </c>
+      <c r="G165" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H165" s="15" t="inlineStr">
+        <is>
+          <t>X/Tn</t>
+        </is>
+      </c>
+      <c r="I165" s="10" t="inlineStr">
+        <is>
+          <t>T/Tn</t>
+        </is>
+      </c>
+      <c r="J165" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K165" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L165" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M165" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N165" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O165" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P165" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q165" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R165" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S165" s="2" t="inlineStr">
+        <is>
+          <t>BR-18-04, BR-18-05, BR-18-06, BR-18-11</t>
+        </is>
+      </c>
+      <c r="T165" s="2" t="inlineStr">
+        <is>
+          <t>`PUT /api/v1/ui/forms/{key}/versions/{v}`, `.../test-runs`</t>
+        </is>
+      </c>
+      <c r="U165" s="2" t="inlineStr">
+        <is>
+          <t>SCR-1802 Quyền: `tenant_admin`; AC-03 khi biểu mẫu gắn Policy Pack</t>
+        </is>
+      </c>
+      <c r="V165" s="2" t="inlineStr"/>
+    </row>
+    <row r="166">
+      <c r="A166" s="9" t="inlineStr">
+        <is>
+          <t>QT-18</t>
+        </is>
+      </c>
+      <c r="B166" s="9" t="inlineStr">
+        <is>
+          <t>SCR-1802</t>
+        </is>
+      </c>
+      <c r="C166" s="2" t="inlineStr">
+        <is>
+          <t>Trình dựng biểu mẫu động</t>
+        </is>
+      </c>
+      <c r="D166" s="2" t="inlineStr">
+        <is>
+          <t>SCR-1802.dua-vao-pack</t>
+        </is>
+      </c>
+      <c r="E166" s="2" t="inlineStr">
+        <is>
+          <t>Đưa biểu mẫu vào UI Pack nháp</t>
+        </is>
+      </c>
+      <c r="F166" s="9" t="inlineStr">
+        <is>
+          <t>Có</t>
+        </is>
+      </c>
+      <c r="G166" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H166" s="15" t="inlineStr">
+        <is>
+          <t>X/Tn</t>
+        </is>
+      </c>
+      <c r="I166" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J166" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K166" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L166" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M166" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N166" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O166" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P166" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q166" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R166" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S166" s="2" t="inlineStr"/>
+      <c r="T166" s="2" t="inlineStr">
+        <is>
+          <t>`POST /api/v1/ui/packs/{id}/versions/{v}/forms`</t>
+        </is>
+      </c>
+      <c r="U166" s="2" t="inlineStr">
+        <is>
+          <t>SCR-1802</t>
+        </is>
+      </c>
+      <c r="V166" s="2" t="inlineStr"/>
+    </row>
+    <row r="167">
+      <c r="A167" s="9" t="inlineStr">
+        <is>
+          <t>QT-18</t>
+        </is>
+      </c>
+      <c r="B167" s="9" t="inlineStr">
+        <is>
+          <t>SCR-1803</t>
+        </is>
+      </c>
+      <c r="C167" s="2" t="inlineStr">
+        <is>
+          <t>Chế độ Đảng viên cao tuổi (di động)</t>
+        </is>
+      </c>
+      <c r="D167" s="2" t="inlineStr">
+        <is>
+          <t>SCR-1803.dd</t>
+        </is>
+      </c>
+      <c r="E167" s="2" t="inlineStr">
+        <is>
+          <t>[Di động] Chế độ cao tuổi: xác nhận sinh hoạt, tự đánh giá rút gọn, nhập giọng nói</t>
+        </is>
+      </c>
+      <c r="F167" s="9" t="inlineStr">
+        <is>
+          <t>Di động</t>
+        </is>
+      </c>
+      <c r="G167" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H167" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I167" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J167" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K167" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L167" s="10" t="inlineStr">
+        <is>
+          <t>T/B</t>
+        </is>
+      </c>
+      <c r="M167" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N167" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O167" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P167" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q167" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R167" s="18" t="inlineStr">
+        <is>
+          <t>A*</t>
+        </is>
+      </c>
+      <c r="S167" s="2" t="inlineStr"/>
+      <c r="T167" s="2" t="inlineStr">
+        <is>
           <t>`POST /api/v1/tasks/{id}/progress`, `PUT .../self-assessment`, `/api/v1/ai/speech-to-text`</t>
         </is>
       </c>
-      <c r="U157" s="2" t="inlineStr">
+      <c r="U167" s="2" t="inlineStr">
         <is>
           <t>SCR-1803</t>
         </is>
       </c>
-      <c r="V157" s="2" t="inlineStr"/>
+      <c r="V167" s="2" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:V157"/>
+  <autoFilter ref="A1:V167"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -20745,7 +21837,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H31"/>
+  <dimension ref="A1:H33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -22000,8 +23092,88 @@
         </is>
       </c>
     </row>
+    <row r="32">
+      <c r="A32" s="9" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>SCR-1505</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>Phê duyệt phát hành mẫu luồng</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>Bốn mắt</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>Người phê duyệt (`second_approver`) phải khác người soạn (`wf_template_author`); phiên AAL2 và step-up khi ký gói mẫu.</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>BS-01 SCR-1505</t>
+        </is>
+      </c>
+      <c r="G32" s="2" t="inlineStr">
+        <is>
+          <t>Repo mẫu luồng (merge request), SVC-06</t>
+        </is>
+      </c>
+      <c r="H32" s="2" t="inlineStr">
+        <is>
+          <t>Chưa có MSG (cần bổ sung)</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="9" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>SCR-1506</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>Chuyển người xử lý, gia hạn bước</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>Giới hạn thao tác</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>Chỉ chuyển người xử lý và gia hạn; không sửa biến tiến trình, không nhảy bước; mọi thao tác ghi sổ cái.</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>BS-01 SCR-1506</t>
+        </is>
+      </c>
+      <c r="G33" s="2" t="inlineStr">
+        <is>
+          <t>SVC-06, SVC-09</t>
+        </is>
+      </c>
+      <c r="H33" s="2" t="inlineStr">
+        <is>
+          <t>Chưa có MSG (cần bổ sung)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H31"/>
+  <autoFilter ref="A1:H33"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
QA-05: quyền đọc của quản trị nghiệp vụ, quản trị nền tảng không cần phân công, trang kế hoạch quý trống
- Bốn thao tác đọc giao diện ở /ui (getCurrentUiPack, getHomeLayout,
  getEffectiveFeatureFlags, getCurrentUiForm) chuyển sang dòng API "ui" của
  ma trận; ma trận thêm ô suy luận AC-03 GET cho config và periods.
  OPA: ca kiểm thử mới, 113/113; OpaAuthzIT có ca đọc của AC-03.
- Bộ sinh ma trận xuất PLATFORM_SCOPE_ROLES; SessionService cho vai trò phạm
  vi nền tảng vào làm việc khi không có phân công đơn vị.
- SCR-0402 (QT-04): đơn vị chưa có kế hoạch thì báo trống, người lập chọn kỳ
  quý đang mở rồi lập kế hoạch (createPlan, POST /plans); PlanApi.create và
  giả lập POST /plans (409 TASK-409-PLAN-EXISTS).
- Wiki 14, 15a.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018FJ4b4cYJJ1Ybgq8kKDxxp
</commit_message>
<xml_diff>
--- a/docs/phan-quyen/ma-tran-phan-quyen.xlsx
+++ b/docs/phan-quyen/ma-tran-phan-quyen.xlsx
@@ -21729,7 +21729,7 @@
       </c>
       <c r="E12" s="16" t="inlineStr">
         <is>
-          <t>PUT</t>
+          <t>GET* PUT</t>
         </is>
       </c>
       <c r="F12" s="16" t="inlineStr">
@@ -21779,7 +21779,7 @@
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
-          <t>AC-01 = tenants; AC-02 = bước 4, 5, feature-flags, holiday-calendars; AC-03 = anomaly-thresholds; người dùng khác GET lịch ngày làm việc. AC-02, AC-04 POST còn gồm role-bindings, delegations (SCR-0105, SCR-0107).</t>
+          <t>AC-01 = tenants; AC-02 = bước 4, 5, feature-flags, holiday-calendars; AC-03 = anomaly-thresholds (GET suy luận: đọc bản hiện hành trước khi sửa ở SCR-1401, QA-05 23/10/2026); người dùng khác GET lịch ngày làm việc. AC-02, AC-04 POST còn gồm role-bindings, delegations (SCR-0105, SCR-0107).</t>
         </is>
       </c>
       <c r="P12" s="2" t="inlineStr">
@@ -21805,9 +21805,9 @@
           <t>GET POST</t>
         </is>
       </c>
-      <c r="E13" s="9" t="inlineStr">
-        <is>
-          <t>-</t>
+      <c r="E13" s="13" t="inlineStr">
+        <is>
+          <t>GET*</t>
         </is>
       </c>
       <c r="F13" s="16" t="inlineStr">
@@ -21857,7 +21857,7 @@
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
-          <t>AC-04 POST = approve lệnh; AC-09 POST = duyệt huỷ.</t>
+          <t>AC-04 POST = approve lệnh; AC-09 POST = duyệt huỷ. AC-03 GET (suy luận, QA-05 23/10/2026): chọn kỳ áp dụng khi gửi phê duyệt bộ quy định (BR-15-10) và kỳ của luồng duyệt, ca thử.</t>
         </is>
       </c>
       <c r="P13" s="2" t="inlineStr">

</xml_diff>

<commit_message>
QA-06: AC-09 được gửi duyệt huỷ khoá kỳ; SCR-0801 hiện kết quả hoàn tác
Ma trận API module config thêm POST cho AC-09 khớp chức năng SCR-0801.duyet-huy (BR-08-09), người phụ trách đã đồng ý; sinh lại wiki 15a, quyền giao diện và dữ liệu OPA. currentLockOrder trả lệnh gần nhất khi không còn lệnh chưa huỷ; tác vụ khởi chạy kết thúc DA_HUY không còn báo lỗi. Dev: nhịp worker saga 4 giây. HT-23, HT-24 đạt trên dev (QT-08).

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RAVfcG9eD2dv4ir2E7jhAG
</commit_message>
<xml_diff>
--- a/docs/phan-quyen/ma-tran-phan-quyen.xlsx
+++ b/docs/phan-quyen/ma-tran-phan-quyen.xlsx
@@ -21757,16 +21757,16 @@
           <t>GET</t>
         </is>
       </c>
-      <c r="K12" s="14" t="inlineStr">
+      <c r="K12" s="16" t="inlineStr">
+        <is>
+          <t>GET POST</t>
+        </is>
+      </c>
+      <c r="L12" s="14" t="inlineStr">
         <is>
           <t>GET</t>
         </is>
       </c>
-      <c r="L12" s="14" t="inlineStr">
-        <is>
-          <t>GET</t>
-        </is>
-      </c>
       <c r="M12" s="9" t="inlineStr">
         <is>
           <t>-</t>
@@ -21779,7 +21779,7 @@
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
-          <t>AC-01 = tenants; AC-02 = bước 4, 5, feature-flags, holiday-calendars; AC-03 = anomaly-thresholds (GET suy luận: đọc bản hiện hành trước khi sửa ở SCR-1401, QA-05 23/10/2026); người dùng khác GET lịch ngày làm việc. AC-02, AC-04 POST còn gồm role-bindings, delegations (SCR-0105, SCR-0107).</t>
+          <t>AC-01 = tenants; AC-02 = bước 4, 5, feature-flags, holiday-calendars; AC-03 = anomaly-thresholds (GET suy luận: đọc bản hiện hành trước khi sửa ở SCR-1401, QA-05 23/10/2026); người dùng khác GET lịch ngày làm việc. AC-02, AC-04 POST còn gồm role-bindings, delegations (SCR-0105, SCR-0107). AC-09 POST là duyệt thứ hai huỷ và bù trừ khoá kỳ (SCR-0801.duyet-huy, BR-08-09; QA-06 24/10/2026).</t>
         </is>
       </c>
       <c r="P12" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Phân quyền: hợp đồng phải bao phủ ma trận chức năng; inspector đọc lần đồng bộ
Lượt đo 2 (64 tài khoản) còn một lệch theo màn hình: inspector thấy SCR-0104
nhưng GET /org/sync-runs bị 403 vì org.yaml chỉ ghi tenant_admin. Thêm phép
kiểm kiem_hop_dong_bao_phu_chuc_nang vào gen_matrix.py (chạy ở mọi lệnh),
thêm inspector vào listOrgSyncRuns theo bảng tác nhân TL-02 (AC-10), siết suy
luận: ô R chỉ kéo theo GET nên bỏ PUT* của tenant_admin ở dòng policies; sinh
lại wiki 15a, xlsx, permissions.generated.ts, dữ liệu OPA (opa test 115/115).
QT-01, SCR-0104, YC-PT-21, YC-PT-26.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UcF6NoqDcB9dEtwcbHnM4c
</commit_message>
<xml_diff>
--- a/docs/phan-quyen/ma-tran-phan-quyen.xlsx
+++ b/docs/phan-quyen/ma-tran-phan-quyen.xlsx
@@ -21488,9 +21488,9 @@
           <t>-</t>
         </is>
       </c>
-      <c r="D9" s="18" t="inlineStr">
-        <is>
-          <t>GET* PUT*</t>
+      <c r="D9" s="13" t="inlineStr">
+        <is>
+          <t>GET*</t>
         </is>
       </c>
       <c r="E9" s="16" t="inlineStr">
@@ -21545,7 +21545,7 @@
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>AC-08 POST = approve (TL-02) hoặc publish (TL-01, `policy_approver`). Bổ sung 24/10/2026 (suy luận, YC-PT-21): tenant_admin PUT theo ma trận chức năng (SCR-1501.soan).</t>
+          <t>AC-08 POST = approve (TL-02) hoặc publish (TL-01, `policy_approver`).</t>
         </is>
       </c>
       <c r="P9" s="2" t="inlineStr">

</xml_diff>

<commit_message>
QA: HT-30 cấp listOrgPersons cho appraiser để thẩm định lập được hội nghị kiểm điểm
Hộp thoại "Lập hội nghị" (SCR-1101.tao, AC-07) nạp GET /org/persons để chọn thành phần,
nhưng hợp đồng org.yaml chỉ cấp listOrgPersons cho manager, leader, tenant_admin nên
org-service (ContractPolicyAdapter) trả 403 cho thamdinh. Thêm appraiser (chỉ cộng thêm,
YC-PT-09, ghi wiki 14); cột API của SCR-1101.tao ghi thêm /org/persons và
/dossiers/special-cases để phép kiểm bao phủ giữ chỗ này; sinh lại operation-policies.json
và đầu ra gen_matrix; danh mục HT-30 bổ sung AC-07 (thamdinh).

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KcF1KqAcEP78x5iFSgMFRv
</commit_message>
<xml_diff>
--- a/docs/phan-quyen/ma-tran-phan-quyen.xlsx
+++ b/docs/phan-quyen/ma-tran-phan-quyen.xlsx
@@ -14885,7 +14885,7 @@
       <c r="S125" s="2" t="inlineStr"/>
       <c r="T125" s="2" t="inlineStr">
         <is>
-          <t>`POST /api/v1/dossiers/meetings`</t>
+          <t>`POST /api/v1/dossiers/meetings`, `GET /api/v1/org/persons`, `GET /api/v1/dossiers/special-cases`</t>
         </is>
       </c>
       <c r="U125" s="2" t="inlineStr">
@@ -14895,7 +14895,7 @@
       </c>
       <c r="V125" s="2" t="inlineStr">
         <is>
-          <t>SCR-1101 không có nút tạo; TL-01 ghi `org_officer`, ánh xạ sang AC-07 là suy luận.</t>
+          <t>SCR-1101 không có nút tạo; TL-01 ghi `org_officer`, ánh xạ sang AC-07 là suy luận. Hộp thoại lập hội nghị chọn người được kiểm điểm, chủ trì, thư ký, thành phần qua `GET /org/persons` và hiện trường hợp đặc thù qua `GET /dossiers/special-cases` (HT-30, wiki 14).</t>
         </is>
       </c>
     </row>

</xml_diff>